<commit_message>
Form con el espíritu de la primera colecta: invitación, chiste y foto final
- Textos del Form editables desde la app y guardados en la configuración:
  título, invitación con ¿Cuándo?/¿Dónde?, opciones de asistencia con humor,
  opciones y descripción de rol ("declaración formal de rol").
- Página final para todas las personas (también quienes no van): pregunta
  chiste configurable ("¿Cuál es tu mood financiero? (importantísimo)") y
  despedida con la foto de la comisión (link de Drive o directo).
- Página "Automatización automática de autos" en insumos.
- El botón para guardar la configuración ahora incluye los textos del Form.
- Tests para textos, detección de columnas y la app.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019oe2a6HEDkUfhap1VckAWr
</commit_message>
<xml_diff>
--- a/ejemplos/respuestas_financiamiento_ficticias.xlsx
+++ b/ejemplos/respuestas_financiamiento_ficticias.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S61"/>
+  <dimension ref="A1:T61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -429,22 +429,22 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>Nombre y apellido</t>
+          <t>Nombre completo</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>Teléfono (WhatsApp)</t>
+          <t>Número de teléfono (formato +569XXXXXXXX)</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>¿Cuál es tu rol?</t>
+          <t>¿Eres...? (declaración formal de rol)</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>¿Vas a asistir a la colecta?</t>
+          <t>¿Puedes ir a la colecta?</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
@@ -510,6 +510,11 @@
       <c r="S1" t="inlineStr">
         <is>
           <t>Comentarios</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>¿Cuál es tu mood financiero? (importantísimo)</t>
         </is>
       </c>
     </row>
@@ -536,51 +541,48 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Comisionado/a</t>
+          <t>Comisionadx</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>Sí, voy con todo 🤑</t>
         </is>
       </c>
       <c r="G2" t="inlineStr"/>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>Viernes</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>Viernes</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>Viernes</t>
-        </is>
-      </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>Viernes</t>
-        </is>
-      </c>
+      <c r="H2" t="inlineStr"/>
+      <c r="I2" t="inlineStr"/>
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr"/>
       <c r="L2" t="inlineStr"/>
-      <c r="M2" t="inlineStr"/>
-      <c r="N2" t="inlineStr"/>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>Viernes</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>Viernes</t>
+        </is>
+      </c>
       <c r="O2" t="inlineStr"/>
       <c r="P2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr"/>
       <c r="R2" t="inlineStr">
         <is>
-          <t>Donde me necesiten</t>
+          <t>Los Leones con Eliodoro Yáñez, Tobalaba con El Bosque, Holanda con Pocuro</t>
         </is>
       </c>
       <c r="S2" t="inlineStr"/>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>Depauperada</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -605,59 +607,32 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Staff</t>
+          <t>Comisionadx</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No, odio a financiamiento 😔</t>
         </is>
       </c>
       <c r="G3" t="inlineStr"/>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>Viernes</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>Viernes</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>Viernes</t>
-        </is>
-      </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>Viernes</t>
-        </is>
-      </c>
-      <c r="L3" t="inlineStr">
-        <is>
-          <t>Viernes</t>
-        </is>
-      </c>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>Viernes</t>
-        </is>
-      </c>
+      <c r="H3" t="inlineStr"/>
+      <c r="I3" t="inlineStr"/>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr"/>
+      <c r="L3" t="inlineStr"/>
+      <c r="M3" t="inlineStr"/>
       <c r="N3" t="inlineStr"/>
       <c r="O3" t="inlineStr"/>
-      <c r="P3" t="inlineStr">
-        <is>
-          <t>Sin límite</t>
-        </is>
-      </c>
+      <c r="P3" t="inlineStr"/>
       <c r="Q3" t="inlineStr"/>
-      <c r="R3" t="inlineStr">
-        <is>
-          <t>Donde me necesiten</t>
-        </is>
-      </c>
+      <c r="R3" t="inlineStr"/>
       <c r="S3" t="inlineStr"/>
+      <c r="T3" t="inlineStr">
+        <is>
+          <t>Debilitado</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -682,67 +657,32 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Comisionado/a</t>
+          <t>Comisionadx</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No, odio a financiamiento 😔</t>
         </is>
       </c>
       <c r="G4" t="inlineStr"/>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>Viernes</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>Viernes</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>Viernes</t>
-        </is>
-      </c>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>Viernes</t>
-        </is>
-      </c>
+      <c r="H4" t="inlineStr"/>
+      <c r="I4" t="inlineStr"/>
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr"/>
       <c r="L4" t="inlineStr"/>
-      <c r="M4" t="inlineStr">
-        <is>
-          <t>Sábado</t>
-        </is>
-      </c>
-      <c r="N4" t="inlineStr">
-        <is>
-          <t>Sábado</t>
-        </is>
-      </c>
-      <c r="O4" t="inlineStr">
-        <is>
-          <t>Sábado</t>
-        </is>
-      </c>
-      <c r="P4" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="Q4" t="inlineStr">
-        <is>
-          <t>Sin límite</t>
-        </is>
-      </c>
-      <c r="R4" t="inlineStr">
-        <is>
-          <t>Los Leones con Eliodoro Yáñez, Tobalaba con El Bosque</t>
-        </is>
-      </c>
+      <c r="M4" t="inlineStr"/>
+      <c r="N4" t="inlineStr"/>
+      <c r="O4" t="inlineStr"/>
+      <c r="P4" t="inlineStr"/>
+      <c r="Q4" t="inlineStr"/>
+      <c r="R4" t="inlineStr"/>
       <c r="S4" t="inlineStr"/>
+      <c r="T4" t="inlineStr">
+        <is>
+          <t>Destruida</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -772,11 +712,19 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr"/>
-      <c r="H5" t="inlineStr"/>
+          <t>Sí, voy con todo 🤑</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Viernes</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Viernes</t>
+        </is>
+      </c>
       <c r="I5" t="inlineStr"/>
       <c r="J5" t="inlineStr"/>
       <c r="K5" t="inlineStr"/>
@@ -784,10 +732,23 @@
       <c r="M5" t="inlineStr"/>
       <c r="N5" t="inlineStr"/>
       <c r="O5" t="inlineStr"/>
-      <c r="P5" t="inlineStr"/>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
       <c r="Q5" t="inlineStr"/>
-      <c r="R5" t="inlineStr"/>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>Tobalaba con El Bosque, Holanda con Pocuro, Los Leones con Eliodoro Yáñez</t>
+        </is>
+      </c>
       <c r="S5" t="inlineStr"/>
+      <c r="T5" t="inlineStr">
+        <is>
+          <t>Desmejorado</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -812,12 +773,12 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Staff</t>
+          <t>Comisionadx</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>Sí, voy con todo 🤑</t>
         </is>
       </c>
       <c r="G6" t="inlineStr"/>
@@ -833,50 +794,31 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>Viernes, Sábado</t>
-        </is>
-      </c>
-      <c r="K6" t="inlineStr">
-        <is>
-          <t>Viernes, Sábado</t>
-        </is>
-      </c>
-      <c r="L6" t="inlineStr">
-        <is>
-          <t>Viernes, Sábado</t>
-        </is>
-      </c>
-      <c r="M6" t="inlineStr">
-        <is>
-          <t>Sábado</t>
-        </is>
-      </c>
-      <c r="N6" t="inlineStr">
-        <is>
-          <t>Sábado</t>
-        </is>
-      </c>
-      <c r="O6" t="inlineStr">
-        <is>
-          <t>Sábado</t>
-        </is>
-      </c>
+          <t>Viernes</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr"/>
+      <c r="L6" t="inlineStr"/>
+      <c r="M6" t="inlineStr"/>
+      <c r="N6" t="inlineStr"/>
+      <c r="O6" t="inlineStr"/>
       <c r="P6" t="inlineStr">
         <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="Q6" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="Q6" t="inlineStr"/>
       <c r="R6" t="inlineStr">
         <is>
-          <t>Los Leones con Eliodoro Yáñez, Francisco Bilbao con Tobalaba</t>
+          <t>Donde me necesiten</t>
         </is>
       </c>
       <c r="S6" t="inlineStr"/>
+      <c r="T6" t="inlineStr">
+        <is>
+          <t>Desmejorado</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -901,12 +843,12 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Comisionado/a</t>
+          <t>Comisionadx</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>Sí, voy con todo 🤑</t>
         </is>
       </c>
       <c r="G7" t="inlineStr"/>
@@ -918,27 +860,39 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>Sábado</t>
+          <t>Viernes, Sábado</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>Sábado</t>
+          <t>Viernes, Sábado</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>Sábado</t>
+          <t>Viernes, Sábado</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>Sábado</t>
-        </is>
-      </c>
-      <c r="N7" t="inlineStr"/>
-      <c r="O7" t="inlineStr"/>
-      <c r="P7" t="inlineStr"/>
+          <t>Viernes</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>Viernes</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>Viernes</t>
+        </is>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
       <c r="Q7" t="inlineStr">
         <is>
           <t>Sin límite</t>
@@ -946,10 +900,15 @@
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>Tobalaba con El Bosque, Los Leones con Eliodoro Yáñez, Francisco Bilbao con Tobalaba</t>
+          <t>Francisco Bilbao con Tobalaba</t>
         </is>
       </c>
       <c r="S7" t="inlineStr"/>
+      <c r="T7" t="inlineStr">
+        <is>
+          <t>Depauperada</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -974,12 +933,12 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Comisionado/a</t>
+          <t>Comisionadx</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>Sí, voy con todo 🤑</t>
         </is>
       </c>
       <c r="G8" t="inlineStr"/>
@@ -988,41 +947,46 @@
       <c r="J8" t="inlineStr"/>
       <c r="K8" t="inlineStr">
         <is>
-          <t>Viernes</t>
+          <t>Sábado</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>Viernes</t>
+          <t>Sábado</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>Viernes</t>
+          <t>Sábado</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>Viernes</t>
+          <t>Sábado</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>Viernes</t>
-        </is>
-      </c>
-      <c r="P8" t="inlineStr">
+          <t>Sábado</t>
+        </is>
+      </c>
+      <c r="P8" t="inlineStr"/>
+      <c r="Q8" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="Q8" t="inlineStr"/>
       <c r="R8" t="inlineStr">
         <is>
           <t>Francisco Bilbao con Tobalaba</t>
         </is>
       </c>
       <c r="S8" t="inlineStr"/>
+      <c r="T8" t="inlineStr">
+        <is>
+          <t>Demacrada</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1047,12 +1011,12 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Comisionado/a</t>
+          <t>Comisionadx</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>Sí, voy con todo 🤑</t>
         </is>
       </c>
       <c r="G9" t="inlineStr"/>
@@ -1100,6 +1064,11 @@
         </is>
       </c>
       <c r="S9" t="inlineStr"/>
+      <c r="T9" t="inlineStr">
+        <is>
+          <t>Demacrada</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1124,59 +1093,48 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Comisionado/a</t>
+          <t>Comisionadx</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>Sí, voy con todo 🤑</t>
         </is>
       </c>
       <c r="G10" t="inlineStr"/>
       <c r="H10" t="inlineStr"/>
       <c r="I10" t="inlineStr"/>
       <c r="J10" t="inlineStr"/>
-      <c r="K10" t="inlineStr">
-        <is>
-          <t>Viernes</t>
-        </is>
-      </c>
-      <c r="L10" t="inlineStr">
-        <is>
-          <t>Viernes</t>
-        </is>
-      </c>
-      <c r="M10" t="inlineStr">
-        <is>
-          <t>Viernes</t>
-        </is>
-      </c>
+      <c r="K10" t="inlineStr"/>
+      <c r="L10" t="inlineStr"/>
+      <c r="M10" t="inlineStr"/>
       <c r="N10" t="inlineStr">
         <is>
-          <t>Viernes, Sábado</t>
+          <t>Viernes</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>Viernes, Sábado</t>
+          <t>Viernes</t>
         </is>
       </c>
       <c r="P10" t="inlineStr">
         <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="Q10" t="inlineStr">
-        <is>
           <t>3</t>
         </is>
       </c>
+      <c r="Q10" t="inlineStr"/>
       <c r="R10" t="inlineStr">
         <is>
           <t>Francisco Bilbao con Tobalaba, Tobalaba con El Bosque, Los Leones con Eliodoro Yáñez</t>
         </is>
       </c>
       <c r="S10" t="inlineStr"/>
+      <c r="T10" t="inlineStr">
+        <is>
+          <t>Desmedrado</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1201,12 +1159,12 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Comisionado/a</t>
+          <t>Comisionadx</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>Sí, voy con todo 🤑</t>
         </is>
       </c>
       <c r="G11" t="inlineStr"/>
@@ -1262,6 +1220,11 @@
         </is>
       </c>
       <c r="S11" t="inlineStr"/>
+      <c r="T11" t="inlineStr">
+        <is>
+          <t>Demacrada</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1286,51 +1249,64 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Comisionado/a</t>
+          <t>Comisionadx</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="G12" t="inlineStr"/>
-      <c r="H12" t="inlineStr"/>
-      <c r="I12" t="inlineStr"/>
-      <c r="J12" t="inlineStr"/>
+          <t>Sí, voy con todo 🤑</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>Viernes</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Viernes</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>Viernes</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>Viernes</t>
+        </is>
+      </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>Sábado</t>
+          <t>Viernes</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>Sábado</t>
-        </is>
-      </c>
-      <c r="M12" t="inlineStr">
-        <is>
-          <t>Sábado</t>
-        </is>
-      </c>
-      <c r="N12" t="inlineStr">
-        <is>
-          <t>Sábado</t>
-        </is>
-      </c>
+          <t>Viernes</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr"/>
+      <c r="N12" t="inlineStr"/>
       <c r="O12" t="inlineStr"/>
-      <c r="P12" t="inlineStr"/>
-      <c r="Q12" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
+      <c r="P12" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="Q12" t="inlineStr"/>
       <c r="R12" t="inlineStr">
         <is>
-          <t>Francisco Bilbao con Tobalaba</t>
+          <t>Donde me necesiten</t>
         </is>
       </c>
       <c r="S12" t="inlineStr"/>
+      <c r="T12" t="inlineStr">
+        <is>
+          <t>Demacrada</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1355,59 +1331,60 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Comisionado/a</t>
+          <t>Jefx de comisión</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>Sí, voy con todo 🤑</t>
         </is>
       </c>
       <c r="G13" t="inlineStr"/>
-      <c r="H13" t="inlineStr">
-        <is>
-          <t>Viernes</t>
-        </is>
-      </c>
+      <c r="H13" t="inlineStr"/>
       <c r="I13" t="inlineStr">
         <is>
-          <t>Viernes</t>
+          <t>Sábado</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>Viernes</t>
+          <t>Sábado</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>Viernes</t>
+          <t>Sábado</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>Viernes</t>
+          <t>Sábado</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>Viernes</t>
+          <t>Sábado</t>
         </is>
       </c>
       <c r="N13" t="inlineStr"/>
       <c r="O13" t="inlineStr"/>
-      <c r="P13" t="inlineStr">
+      <c r="P13" t="inlineStr"/>
+      <c r="Q13" t="inlineStr">
         <is>
           <t>Sin límite</t>
         </is>
       </c>
-      <c r="Q13" t="inlineStr"/>
       <c r="R13" t="inlineStr">
         <is>
-          <t>Holanda con Pocuro, Tobalaba con El Bosque, Los Leones con Eliodoro Yáñez, Francisco Bilbao con Tobalaba</t>
+          <t>Donde me necesiten</t>
         </is>
       </c>
       <c r="S13" t="inlineStr"/>
+      <c r="T13" t="inlineStr">
+        <is>
+          <t>Depauperada</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1432,47 +1409,52 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Staff</t>
+          <t>Comisionadx</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>Sí, voy con todo 🤑</t>
         </is>
       </c>
       <c r="G14" t="inlineStr"/>
-      <c r="H14" t="inlineStr"/>
-      <c r="I14" t="inlineStr"/>
-      <c r="J14" t="inlineStr"/>
-      <c r="K14" t="inlineStr">
-        <is>
-          <t>Viernes</t>
-        </is>
-      </c>
-      <c r="L14" t="inlineStr">
-        <is>
-          <t>Viernes</t>
-        </is>
-      </c>
-      <c r="M14" t="inlineStr">
-        <is>
-          <t>Viernes</t>
-        </is>
-      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Sábado</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>Sábado</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>Sábado</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr"/>
+      <c r="L14" t="inlineStr"/>
+      <c r="M14" t="inlineStr"/>
       <c r="N14" t="inlineStr"/>
       <c r="O14" t="inlineStr"/>
-      <c r="P14" t="inlineStr">
+      <c r="P14" t="inlineStr"/>
+      <c r="Q14" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="Q14" t="inlineStr"/>
       <c r="R14" t="inlineStr">
         <is>
           <t>Tobalaba con El Bosque, Los Leones con Eliodoro Yáñez, Holanda con Pocuro, Francisco Bilbao con Tobalaba</t>
         </is>
       </c>
       <c r="S14" t="inlineStr"/>
+      <c r="T14" t="inlineStr">
+        <is>
+          <t>Desmedrado</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1502,29 +1484,21 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>Sí, voy con todo 🤑</t>
         </is>
       </c>
       <c r="G15" t="inlineStr"/>
       <c r="H15" t="inlineStr"/>
-      <c r="I15" t="inlineStr">
-        <is>
-          <t>Sábado</t>
-        </is>
-      </c>
-      <c r="J15" t="inlineStr">
-        <is>
-          <t>Sábado</t>
-        </is>
-      </c>
+      <c r="I15" t="inlineStr"/>
+      <c r="J15" t="inlineStr"/>
       <c r="K15" t="inlineStr">
         <is>
-          <t>Viernes, Sábado</t>
+          <t>Sábado</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>Viernes, Sábado</t>
+          <t>Sábado</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
@@ -1538,22 +1512,23 @@
         </is>
       </c>
       <c r="O15" t="inlineStr"/>
-      <c r="P15" t="inlineStr">
+      <c r="P15" t="inlineStr"/>
+      <c r="Q15" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="Q15" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>Donde me necesiten</t>
+          <t>Los Leones con Eliodoro Yáñez, Holanda con Pocuro, Tobalaba con El Bosque</t>
         </is>
       </c>
       <c r="S15" t="inlineStr"/>
+      <c r="T15" t="inlineStr">
+        <is>
+          <t>Desmejorado</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1583,58 +1558,51 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>Sí, voy con todo 🤑</t>
         </is>
       </c>
       <c r="G16" t="inlineStr"/>
       <c r="H16" t="inlineStr"/>
-      <c r="I16" t="inlineStr">
-        <is>
-          <t>Sábado</t>
-        </is>
-      </c>
-      <c r="J16" t="inlineStr">
-        <is>
-          <t>Sábado</t>
-        </is>
-      </c>
-      <c r="K16" t="inlineStr">
-        <is>
-          <t>Sábado</t>
-        </is>
-      </c>
+      <c r="I16" t="inlineStr"/>
+      <c r="J16" t="inlineStr"/>
+      <c r="K16" t="inlineStr"/>
       <c r="L16" t="inlineStr">
         <is>
-          <t>Viernes, Sábado</t>
+          <t>Sábado</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>Viernes</t>
+          <t>Sábado</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>Viernes</t>
-        </is>
-      </c>
-      <c r="O16" t="inlineStr"/>
-      <c r="P16" t="inlineStr">
+          <t>Sábado</t>
+        </is>
+      </c>
+      <c r="O16" t="inlineStr">
+        <is>
+          <t>Sábado</t>
+        </is>
+      </c>
+      <c r="P16" t="inlineStr"/>
+      <c r="Q16" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="Q16" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>Los Leones con Eliodoro Yáñez, Francisco Bilbao con Tobalaba, Holanda con Pocuro, Tobalaba con El Bosque</t>
+          <t>Donde me necesiten</t>
         </is>
       </c>
       <c r="S16" t="inlineStr"/>
+      <c r="T16" t="inlineStr">
+        <is>
+          <t>Depauperada</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1659,17 +1627,21 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Comisionado/a</t>
+          <t>Staff</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>Sí, voy con todo 🤑</t>
         </is>
       </c>
       <c r="G17" t="inlineStr"/>
       <c r="H17" t="inlineStr"/>
-      <c r="I17" t="inlineStr"/>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>Viernes</t>
+        </is>
+      </c>
       <c r="J17" t="inlineStr">
         <is>
           <t>Viernes</t>
@@ -1677,17 +1649,17 @@
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>Viernes, Sábado</t>
+          <t>Viernes</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>Viernes, Sábado</t>
+          <t>Viernes</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>Viernes, Sábado</t>
+          <t>Viernes</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
@@ -1698,20 +1670,21 @@
       <c r="O17" t="inlineStr"/>
       <c r="P17" t="inlineStr">
         <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="Q17" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="Q17" t="inlineStr"/>
       <c r="R17" t="inlineStr">
         <is>
           <t>Donde me necesiten</t>
         </is>
       </c>
       <c r="S17" t="inlineStr"/>
+      <c r="T17" t="inlineStr">
+        <is>
+          <t>Desmejorado</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1736,51 +1709,39 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Staff</t>
+          <t>Familia</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="G18" t="inlineStr">
-        <is>
-          <t>Viernes, Sábado</t>
-        </is>
-      </c>
-      <c r="H18" t="inlineStr">
-        <is>
-          <t>Viernes, Sábado</t>
-        </is>
-      </c>
-      <c r="I18" t="inlineStr">
-        <is>
-          <t>Viernes</t>
-        </is>
-      </c>
-      <c r="J18" t="inlineStr">
-        <is>
-          <t>Viernes</t>
-        </is>
-      </c>
+          <t>Sí, voy con todo 🤑</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr"/>
+      <c r="H18" t="inlineStr"/>
+      <c r="I18" t="inlineStr"/>
+      <c r="J18" t="inlineStr"/>
       <c r="K18" t="inlineStr">
         <is>
-          <t>Viernes</t>
-        </is>
-      </c>
-      <c r="L18" t="inlineStr"/>
-      <c r="M18" t="inlineStr"/>
+          <t>Sábado</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>Sábado</t>
+        </is>
+      </c>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>Sábado</t>
+        </is>
+      </c>
       <c r="N18" t="inlineStr"/>
       <c r="O18" t="inlineStr"/>
-      <c r="P18" t="inlineStr">
-        <is>
-          <t>Sin límite</t>
-        </is>
-      </c>
+      <c r="P18" t="inlineStr"/>
       <c r="Q18" t="inlineStr">
         <is>
-          <t>Sin límite</t>
+          <t>2</t>
         </is>
       </c>
       <c r="R18" t="inlineStr">
@@ -1789,6 +1750,11 @@
         </is>
       </c>
       <c r="S18" t="inlineStr"/>
+      <c r="T18" t="inlineStr">
+        <is>
+          <t>Debilitado</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1813,12 +1779,12 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Comisionado/a</t>
+          <t>Staff</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí, voy con todo 🤑</t>
         </is>
       </c>
       <c r="G19" t="inlineStr"/>
@@ -1828,12 +1794,37 @@
       <c r="K19" t="inlineStr"/>
       <c r="L19" t="inlineStr"/>
       <c r="M19" t="inlineStr"/>
-      <c r="N19" t="inlineStr"/>
-      <c r="O19" t="inlineStr"/>
-      <c r="P19" t="inlineStr"/>
-      <c r="Q19" t="inlineStr"/>
-      <c r="R19" t="inlineStr"/>
+      <c r="N19" t="inlineStr">
+        <is>
+          <t>Viernes, Sábado</t>
+        </is>
+      </c>
+      <c r="O19" t="inlineStr">
+        <is>
+          <t>Viernes, Sábado</t>
+        </is>
+      </c>
+      <c r="P19" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="Q19" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R19" t="inlineStr">
+        <is>
+          <t>Donde me necesiten</t>
+        </is>
+      </c>
       <c r="S19" t="inlineStr"/>
+      <c r="T19" t="inlineStr">
+        <is>
+          <t>Demacrada</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1858,12 +1849,12 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Familia</t>
+          <t>Comisionadx</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>Sí, voy con todo 🤑</t>
         </is>
       </c>
       <c r="G20" t="inlineStr"/>
@@ -1875,7 +1866,7 @@
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>Sábado</t>
+          <t>Viernes, Sábado</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
@@ -1890,19 +1881,11 @@
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>Viernes, Sábado</t>
-        </is>
-      </c>
-      <c r="N20" t="inlineStr">
-        <is>
-          <t>Viernes</t>
-        </is>
-      </c>
-      <c r="O20" t="inlineStr">
-        <is>
-          <t>Viernes</t>
-        </is>
-      </c>
+          <t>Sábado</t>
+        </is>
+      </c>
+      <c r="N20" t="inlineStr"/>
+      <c r="O20" t="inlineStr"/>
       <c r="P20" t="inlineStr">
         <is>
           <t>2</t>
@@ -1919,6 +1902,11 @@
         </is>
       </c>
       <c r="S20" t="inlineStr"/>
+      <c r="T20" t="inlineStr">
+        <is>
+          <t>Desmejorado</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1943,51 +1931,56 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Familia</t>
+          <t>Jefx de comisión</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="G21" t="inlineStr"/>
-      <c r="H21" t="inlineStr"/>
+          <t>Sí, voy con todo 🤑</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>Viernes</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>Viernes</t>
+        </is>
+      </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>Sábado</t>
+          <t>Viernes</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>Sábado</t>
-        </is>
-      </c>
-      <c r="K21" t="inlineStr">
-        <is>
-          <t>Sábado</t>
-        </is>
-      </c>
-      <c r="L21" t="inlineStr">
-        <is>
-          <t>Sábado</t>
-        </is>
-      </c>
+          <t>Viernes</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr"/>
+      <c r="L21" t="inlineStr"/>
       <c r="M21" t="inlineStr"/>
       <c r="N21" t="inlineStr"/>
       <c r="O21" t="inlineStr"/>
-      <c r="P21" t="inlineStr"/>
-      <c r="Q21" t="inlineStr">
+      <c r="P21" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
+      <c r="Q21" t="inlineStr"/>
       <c r="R21" t="inlineStr">
         <is>
-          <t>Los Leones con Eliodoro Yáñez, Tobalaba con El Bosque, Holanda con Pocuro, Francisco Bilbao con Tobalaba</t>
+          <t>Tobalaba con El Bosque, Holanda con Pocuro</t>
         </is>
       </c>
       <c r="S21" t="inlineStr"/>
+      <c r="T21" t="inlineStr">
+        <is>
+          <t>Desmejorado</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -2017,7 +2010,7 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>Sí, voy con todo 🤑</t>
         </is>
       </c>
       <c r="G22" t="inlineStr"/>
@@ -2042,21 +2035,34 @@
           <t>Viernes</t>
         </is>
       </c>
-      <c r="M22" t="inlineStr"/>
-      <c r="N22" t="inlineStr"/>
+      <c r="M22" t="inlineStr">
+        <is>
+          <t>Viernes</t>
+        </is>
+      </c>
+      <c r="N22" t="inlineStr">
+        <is>
+          <t>Viernes</t>
+        </is>
+      </c>
       <c r="O22" t="inlineStr"/>
       <c r="P22" t="inlineStr">
         <is>
-          <t>Sin límite</t>
+          <t>3</t>
         </is>
       </c>
       <c r="Q22" t="inlineStr"/>
       <c r="R22" t="inlineStr">
         <is>
-          <t>Donde me necesiten</t>
+          <t>Francisco Bilbao con Tobalaba, Holanda con Pocuro, Los Leones con Eliodoro Yáñez, Tobalaba con El Bosque</t>
         </is>
       </c>
       <c r="S22" t="inlineStr"/>
+      <c r="T22" t="inlineStr">
+        <is>
+          <t>Debilitado</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -2081,19 +2087,31 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Comisionado/a</t>
+          <t>Comisionadx</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>Sí, voy con todo 🤑</t>
         </is>
       </c>
       <c r="G23" t="inlineStr"/>
       <c r="H23" t="inlineStr"/>
-      <c r="I23" t="inlineStr"/>
-      <c r="J23" t="inlineStr"/>
-      <c r="K23" t="inlineStr"/>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>Sábado</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>Sábado</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>Sábado</t>
+        </is>
+      </c>
       <c r="L23" t="inlineStr">
         <is>
           <t>Sábado</t>
@@ -2104,32 +2122,25 @@
           <t>Sábado</t>
         </is>
       </c>
-      <c r="N23" t="inlineStr">
-        <is>
-          <t>Viernes, Sábado</t>
-        </is>
-      </c>
-      <c r="O23" t="inlineStr">
-        <is>
-          <t>Viernes, Sábado</t>
-        </is>
-      </c>
-      <c r="P23" t="inlineStr">
+      <c r="N23" t="inlineStr"/>
+      <c r="O23" t="inlineStr"/>
+      <c r="P23" t="inlineStr"/>
+      <c r="Q23" t="inlineStr">
         <is>
           <t>Sin límite</t>
         </is>
       </c>
-      <c r="Q23" t="inlineStr">
-        <is>
-          <t>Sin límite</t>
-        </is>
-      </c>
       <c r="R23" t="inlineStr">
         <is>
           <t>Donde me necesiten</t>
         </is>
       </c>
       <c r="S23" t="inlineStr"/>
+      <c r="T23" t="inlineStr">
+        <is>
+          <t>Demacrada</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -2154,12 +2165,12 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Comisionado/a</t>
+          <t>Comisionadx</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>Sí, voy con todo 🤑</t>
         </is>
       </c>
       <c r="G24" t="inlineStr"/>
@@ -2176,33 +2187,26 @@
       <c r="J24" t="inlineStr"/>
       <c r="K24" t="inlineStr"/>
       <c r="L24" t="inlineStr"/>
-      <c r="M24" t="inlineStr">
-        <is>
-          <t>Sábado</t>
-        </is>
-      </c>
-      <c r="N24" t="inlineStr">
-        <is>
-          <t>Sábado</t>
-        </is>
-      </c>
+      <c r="M24" t="inlineStr"/>
+      <c r="N24" t="inlineStr"/>
       <c r="O24" t="inlineStr"/>
       <c r="P24" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="Q24" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+      <c r="Q24" t="inlineStr"/>
       <c r="R24" t="inlineStr">
         <is>
-          <t>Francisco Bilbao con Tobalaba, Los Leones con Eliodoro Yáñez, Holanda con Pocuro, Tobalaba con El Bosque</t>
+          <t>Donde me necesiten</t>
         </is>
       </c>
       <c r="S24" t="inlineStr"/>
+      <c r="T24" t="inlineStr">
+        <is>
+          <t>Depauperada</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -2227,17 +2231,29 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Staff</t>
+          <t>Jefx de comisión</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="G25" t="inlineStr"/>
-      <c r="H25" t="inlineStr"/>
-      <c r="I25" t="inlineStr"/>
+          <t>Sí, voy con todo 🤑</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>Sábado</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>Sábado</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>Sábado</t>
+        </is>
+      </c>
       <c r="J25" t="inlineStr">
         <is>
           <t>Sábado</t>
@@ -2248,34 +2264,31 @@
           <t>Sábado</t>
         </is>
       </c>
-      <c r="L25" t="inlineStr"/>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>Sábado</t>
+        </is>
+      </c>
       <c r="M25" t="inlineStr"/>
-      <c r="N25" t="inlineStr">
-        <is>
-          <t>Viernes</t>
-        </is>
-      </c>
-      <c r="O25" t="inlineStr">
-        <is>
-          <t>Viernes</t>
-        </is>
-      </c>
-      <c r="P25" t="inlineStr">
+      <c r="N25" t="inlineStr"/>
+      <c r="O25" t="inlineStr"/>
+      <c r="P25" t="inlineStr"/>
+      <c r="Q25" t="inlineStr">
         <is>
           <t>Sin límite</t>
         </is>
       </c>
-      <c r="Q25" t="inlineStr">
-        <is>
-          <t>Sin límite</t>
-        </is>
-      </c>
       <c r="R25" t="inlineStr">
         <is>
-          <t>Donde me necesiten</t>
+          <t>Francisco Bilbao con Tobalaba</t>
         </is>
       </c>
       <c r="S25" t="inlineStr"/>
+      <c r="T25" t="inlineStr">
+        <is>
+          <t>Demacrada</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -2300,47 +2313,64 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Familia</t>
+          <t>Staff</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>Sí, voy con todo 🤑</t>
         </is>
       </c>
       <c r="G26" t="inlineStr"/>
-      <c r="H26" t="inlineStr">
-        <is>
-          <t>Sábado</t>
-        </is>
-      </c>
-      <c r="I26" t="inlineStr">
-        <is>
-          <t>Sábado</t>
-        </is>
-      </c>
+      <c r="H26" t="inlineStr"/>
+      <c r="I26" t="inlineStr"/>
       <c r="J26" t="inlineStr">
         <is>
-          <t>Sábado</t>
-        </is>
-      </c>
-      <c r="K26" t="inlineStr"/>
-      <c r="L26" t="inlineStr"/>
-      <c r="M26" t="inlineStr"/>
-      <c r="N26" t="inlineStr"/>
+          <t>Viernes</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>Viernes</t>
+        </is>
+      </c>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>Viernes, Sábado</t>
+        </is>
+      </c>
+      <c r="M26" t="inlineStr">
+        <is>
+          <t>Viernes, Sábado</t>
+        </is>
+      </c>
+      <c r="N26" t="inlineStr">
+        <is>
+          <t>Viernes, Sábado</t>
+        </is>
+      </c>
       <c r="O26" t="inlineStr"/>
-      <c r="P26" t="inlineStr"/>
+      <c r="P26" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="Q26" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>Sin límite</t>
         </is>
       </c>
       <c r="R26" t="inlineStr">
         <is>
-          <t>Los Leones con Eliodoro Yáñez, Tobalaba con El Bosque, Holanda con Pocuro, Francisco Bilbao con Tobalaba</t>
+          <t>Donde me necesiten</t>
         </is>
       </c>
       <c r="S26" t="inlineStr"/>
+      <c r="T26" t="inlineStr">
+        <is>
+          <t>Debilitado</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -2365,51 +2395,60 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Comisionado/a</t>
+          <t>Familia</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="G27" t="inlineStr">
-        <is>
-          <t>Sábado</t>
-        </is>
-      </c>
+          <t>Sí, voy con todo 🤑</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr"/>
       <c r="H27" t="inlineStr">
         <is>
-          <t>Sábado</t>
+          <t>Viernes</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>Sábado</t>
+          <t>Viernes</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>Sábado</t>
-        </is>
-      </c>
-      <c r="K27" t="inlineStr"/>
-      <c r="L27" t="inlineStr"/>
+          <t>Viernes</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>Viernes</t>
+        </is>
+      </c>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>Viernes</t>
+        </is>
+      </c>
       <c r="M27" t="inlineStr"/>
       <c r="N27" t="inlineStr"/>
       <c r="O27" t="inlineStr"/>
-      <c r="P27" t="inlineStr"/>
-      <c r="Q27" t="inlineStr">
+      <c r="P27" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
+      <c r="Q27" t="inlineStr"/>
       <c r="R27" t="inlineStr">
         <is>
           <t>Donde me necesiten</t>
         </is>
       </c>
       <c r="S27" t="inlineStr"/>
+      <c r="T27" t="inlineStr">
+        <is>
+          <t>Desmejorado</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -2434,27 +2473,68 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Familia</t>
+          <t>Comisionadx</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G28" t="inlineStr"/>
-      <c r="H28" t="inlineStr"/>
-      <c r="I28" t="inlineStr"/>
-      <c r="J28" t="inlineStr"/>
-      <c r="K28" t="inlineStr"/>
-      <c r="L28" t="inlineStr"/>
+          <t>Sí, voy con todo 🤑</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>Sábado</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>Sábado</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>Viernes, Sábado</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>Viernes, Sábado</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>Viernes, Sábado</t>
+        </is>
+      </c>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>Viernes</t>
+        </is>
+      </c>
       <c r="M28" t="inlineStr"/>
       <c r="N28" t="inlineStr"/>
       <c r="O28" t="inlineStr"/>
-      <c r="P28" t="inlineStr"/>
-      <c r="Q28" t="inlineStr"/>
-      <c r="R28" t="inlineStr"/>
+      <c r="P28" t="inlineStr">
+        <is>
+          <t>Sin límite</t>
+        </is>
+      </c>
+      <c r="Q28" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="R28" t="inlineStr">
+        <is>
+          <t>Donde me necesiten</t>
+        </is>
+      </c>
       <c r="S28" t="inlineStr"/>
+      <c r="T28" t="inlineStr">
+        <is>
+          <t>Debilitado</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -2479,51 +2559,32 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Comisionado/a</t>
+          <t>Jefx de comisión</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No, odio a financiamiento 😔</t>
         </is>
       </c>
       <c r="G29" t="inlineStr"/>
       <c r="H29" t="inlineStr"/>
       <c r="I29" t="inlineStr"/>
       <c r="J29" t="inlineStr"/>
-      <c r="K29" t="inlineStr">
-        <is>
-          <t>Sábado</t>
-        </is>
-      </c>
-      <c r="L29" t="inlineStr">
-        <is>
-          <t>Sábado</t>
-        </is>
-      </c>
-      <c r="M29" t="inlineStr">
-        <is>
-          <t>Sábado</t>
-        </is>
-      </c>
-      <c r="N29" t="inlineStr">
-        <is>
-          <t>Sábado</t>
-        </is>
-      </c>
+      <c r="K29" t="inlineStr"/>
+      <c r="L29" t="inlineStr"/>
+      <c r="M29" t="inlineStr"/>
+      <c r="N29" t="inlineStr"/>
       <c r="O29" t="inlineStr"/>
       <c r="P29" t="inlineStr"/>
-      <c r="Q29" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="R29" t="inlineStr">
-        <is>
-          <t>Holanda con Pocuro, Los Leones con Eliodoro Yáñez, Francisco Bilbao con Tobalaba</t>
-        </is>
-      </c>
+      <c r="Q29" t="inlineStr"/>
+      <c r="R29" t="inlineStr"/>
       <c r="S29" t="inlineStr"/>
+      <c r="T29" t="inlineStr">
+        <is>
+          <t>Destruida</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -2548,21 +2609,17 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Familia</t>
+          <t>Jefx de comisión</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>Sí, voy con todo 🤑</t>
         </is>
       </c>
       <c r="G30" t="inlineStr"/>
       <c r="H30" t="inlineStr"/>
-      <c r="I30" t="inlineStr">
-        <is>
-          <t>Viernes</t>
-        </is>
-      </c>
+      <c r="I30" t="inlineStr"/>
       <c r="J30" t="inlineStr">
         <is>
           <t>Viernes</t>
@@ -2570,45 +2627,50 @@
       </c>
       <c r="K30" t="inlineStr">
         <is>
+          <t>Viernes</t>
+        </is>
+      </c>
+      <c r="L30" t="inlineStr">
+        <is>
           <t>Viernes, Sábado</t>
         </is>
       </c>
-      <c r="L30" t="inlineStr">
+      <c r="M30" t="inlineStr">
         <is>
           <t>Viernes, Sábado</t>
         </is>
       </c>
-      <c r="M30" t="inlineStr">
-        <is>
-          <t>Sábado</t>
-        </is>
-      </c>
       <c r="N30" t="inlineStr">
         <is>
-          <t>Sábado</t>
+          <t>Viernes, Sábado</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>Sábado</t>
+          <t>Viernes, Sábado</t>
         </is>
       </c>
       <c r="P30" t="inlineStr">
         <is>
-          <t>Sin límite</t>
+          <t>2</t>
         </is>
       </c>
       <c r="Q30" t="inlineStr">
         <is>
-          <t>Sin límite</t>
+          <t>3</t>
         </is>
       </c>
       <c r="R30" t="inlineStr">
         <is>
-          <t>Tobalaba con El Bosque, Holanda con Pocuro, Francisco Bilbao con Tobalaba</t>
+          <t>Tobalaba con El Bosque, Los Leones con Eliodoro Yáñez, Holanda con Pocuro</t>
         </is>
       </c>
       <c r="S30" t="inlineStr"/>
+      <c r="T30" t="inlineStr">
+        <is>
+          <t>Destruida</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -2633,51 +2695,56 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Staff</t>
+          <t>Familia</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>Sí, voy con todo 🤑</t>
         </is>
       </c>
       <c r="G31" t="inlineStr"/>
       <c r="H31" t="inlineStr"/>
       <c r="I31" t="inlineStr"/>
-      <c r="J31" t="inlineStr">
-        <is>
-          <t>Viernes</t>
-        </is>
-      </c>
-      <c r="K31" t="inlineStr">
-        <is>
-          <t>Viernes</t>
-        </is>
-      </c>
+      <c r="J31" t="inlineStr"/>
+      <c r="K31" t="inlineStr"/>
       <c r="L31" t="inlineStr">
         <is>
-          <t>Viernes</t>
+          <t>Sábado</t>
         </is>
       </c>
       <c r="M31" t="inlineStr">
         <is>
-          <t>Viernes</t>
-        </is>
-      </c>
-      <c r="N31" t="inlineStr"/>
-      <c r="O31" t="inlineStr"/>
-      <c r="P31" t="inlineStr">
-        <is>
-          <t>Sin límite</t>
-        </is>
-      </c>
-      <c r="Q31" t="inlineStr"/>
+          <t>Sábado</t>
+        </is>
+      </c>
+      <c r="N31" t="inlineStr">
+        <is>
+          <t>Sábado</t>
+        </is>
+      </c>
+      <c r="O31" t="inlineStr">
+        <is>
+          <t>Sábado</t>
+        </is>
+      </c>
+      <c r="P31" t="inlineStr"/>
+      <c r="Q31" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="R31" t="inlineStr">
         <is>
-          <t>Donde me necesiten</t>
+          <t>Holanda con Pocuro</t>
         </is>
       </c>
       <c r="S31" t="inlineStr"/>
+      <c r="T31" t="inlineStr">
+        <is>
+          <t>Desmejorado</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -2702,17 +2769,25 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Familia</t>
+          <t>Jefx de comisión</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>Sí, voy con todo 🤑</t>
         </is>
       </c>
       <c r="G32" t="inlineStr"/>
-      <c r="H32" t="inlineStr"/>
-      <c r="I32" t="inlineStr"/>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>Sábado</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>Sábado</t>
+        </is>
+      </c>
       <c r="J32" t="inlineStr">
         <is>
           <t>Sábado</t>
@@ -2734,15 +2809,20 @@
       <c r="P32" t="inlineStr"/>
       <c r="Q32" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>Sin límite</t>
         </is>
       </c>
       <c r="R32" t="inlineStr">
         <is>
-          <t>Donde me necesiten</t>
+          <t>Holanda con Pocuro, Tobalaba con El Bosque</t>
         </is>
       </c>
       <c r="S32" t="inlineStr"/>
+      <c r="T32" t="inlineStr">
+        <is>
+          <t>Destruida</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -2772,54 +2852,51 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>Sí, voy con todo 🤑</t>
         </is>
       </c>
       <c r="G33" t="inlineStr"/>
       <c r="H33" t="inlineStr"/>
       <c r="I33" t="inlineStr"/>
-      <c r="J33" t="inlineStr">
-        <is>
-          <t>Viernes</t>
-        </is>
-      </c>
-      <c r="K33" t="inlineStr">
-        <is>
-          <t>Viernes</t>
-        </is>
-      </c>
+      <c r="J33" t="inlineStr"/>
+      <c r="K33" t="inlineStr"/>
       <c r="L33" t="inlineStr">
         <is>
-          <t>Viernes</t>
+          <t>Sábado</t>
         </is>
       </c>
       <c r="M33" t="inlineStr">
         <is>
-          <t>Viernes</t>
+          <t>Sábado</t>
         </is>
       </c>
       <c r="N33" t="inlineStr">
         <is>
-          <t>Viernes</t>
+          <t>Sábado</t>
         </is>
       </c>
       <c r="O33" t="inlineStr">
         <is>
-          <t>Viernes</t>
-        </is>
-      </c>
-      <c r="P33" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="Q33" t="inlineStr"/>
+          <t>Sábado</t>
+        </is>
+      </c>
+      <c r="P33" t="inlineStr"/>
+      <c r="Q33" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
       <c r="R33" t="inlineStr">
         <is>
-          <t>Donde me necesiten</t>
+          <t>Tobalaba con El Bosque</t>
         </is>
       </c>
       <c r="S33" t="inlineStr"/>
+      <c r="T33" t="inlineStr">
+        <is>
+          <t>Depauperada</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -2844,12 +2921,12 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Comisionado/a</t>
+          <t>Comisionadx</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>Sí, voy con todo 🤑</t>
         </is>
       </c>
       <c r="G34" t="inlineStr"/>
@@ -2893,6 +2970,11 @@
         </is>
       </c>
       <c r="S34" t="inlineStr"/>
+      <c r="T34" t="inlineStr">
+        <is>
+          <t>Destruida</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -2917,37 +2999,33 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Familia</t>
+          <t>Jefx de comisión</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="G35" t="inlineStr">
-        <is>
-          <t>Sábado</t>
-        </is>
-      </c>
+          <t>Sí, voy con todo 🤑</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr"/>
       <c r="H35" t="inlineStr">
         <is>
-          <t>Viernes, Sábado</t>
+          <t>Viernes</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>Viernes, Sábado</t>
+          <t>Viernes</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>Viernes, Sábado</t>
+          <t>Viernes</t>
         </is>
       </c>
       <c r="K35" t="inlineStr">
         <is>
-          <t>Viernes, Sábado</t>
+          <t>Viernes</t>
         </is>
       </c>
       <c r="L35" t="inlineStr">
@@ -2963,17 +3041,18 @@
           <t>2</t>
         </is>
       </c>
-      <c r="Q35" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+      <c r="Q35" t="inlineStr"/>
       <c r="R35" t="inlineStr">
         <is>
-          <t>Los Leones con Eliodoro Yáñez</t>
+          <t>Francisco Bilbao con Tobalaba, Holanda con Pocuro, Tobalaba con El Bosque, Los Leones con Eliodoro Yáñez</t>
         </is>
       </c>
       <c r="S35" t="inlineStr"/>
+      <c r="T35" t="inlineStr">
+        <is>
+          <t>Demacrada</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -2998,12 +3077,12 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Comisionado/a</t>
+          <t>Comisionadx</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>Sí, voy con todo 🤑</t>
         </is>
       </c>
       <c r="G36" t="inlineStr"/>
@@ -3047,6 +3126,11 @@
         </is>
       </c>
       <c r="S36" t="inlineStr"/>
+      <c r="T36" t="inlineStr">
+        <is>
+          <t>Depauperada</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -3071,34 +3155,38 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Comisionado/a</t>
+          <t>Comisionadx</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>Sí, voy con todo 🤑</t>
         </is>
       </c>
       <c r="G37" t="inlineStr"/>
       <c r="H37" t="inlineStr"/>
-      <c r="I37" t="inlineStr">
-        <is>
-          <t>Viernes</t>
-        </is>
-      </c>
-      <c r="J37" t="inlineStr">
-        <is>
-          <t>Viernes</t>
-        </is>
-      </c>
+      <c r="I37" t="inlineStr"/>
+      <c r="J37" t="inlineStr"/>
       <c r="K37" t="inlineStr">
         <is>
           <t>Viernes</t>
         </is>
       </c>
-      <c r="L37" t="inlineStr"/>
-      <c r="M37" t="inlineStr"/>
-      <c r="N37" t="inlineStr"/>
+      <c r="L37" t="inlineStr">
+        <is>
+          <t>Viernes</t>
+        </is>
+      </c>
+      <c r="M37" t="inlineStr">
+        <is>
+          <t>Viernes</t>
+        </is>
+      </c>
+      <c r="N37" t="inlineStr">
+        <is>
+          <t>Viernes</t>
+        </is>
+      </c>
       <c r="O37" t="inlineStr"/>
       <c r="P37" t="inlineStr">
         <is>
@@ -3112,6 +3200,11 @@
         </is>
       </c>
       <c r="S37" t="inlineStr"/>
+      <c r="T37" t="inlineStr">
+        <is>
+          <t>Depauperada</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -3141,58 +3234,51 @@
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>Sí, voy con todo 🤑</t>
         </is>
       </c>
       <c r="G38" t="inlineStr"/>
-      <c r="H38" t="inlineStr">
-        <is>
-          <t>Sábado</t>
-        </is>
-      </c>
-      <c r="I38" t="inlineStr">
-        <is>
-          <t>Sábado</t>
-        </is>
-      </c>
+      <c r="H38" t="inlineStr"/>
+      <c r="I38" t="inlineStr"/>
       <c r="J38" t="inlineStr"/>
       <c r="K38" t="inlineStr">
         <is>
-          <t>Viernes</t>
+          <t>Sábado</t>
         </is>
       </c>
       <c r="L38" t="inlineStr">
         <is>
-          <t>Viernes</t>
+          <t>Sábado</t>
         </is>
       </c>
       <c r="M38" t="inlineStr">
         <is>
-          <t>Viernes</t>
+          <t>Sábado</t>
         </is>
       </c>
       <c r="N38" t="inlineStr">
         <is>
-          <t>Viernes</t>
+          <t>Sábado</t>
         </is>
       </c>
       <c r="O38" t="inlineStr"/>
-      <c r="P38" t="inlineStr">
+      <c r="P38" t="inlineStr"/>
+      <c r="Q38" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="Q38" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
       <c r="R38" t="inlineStr">
         <is>
-          <t>Francisco Bilbao con Tobalaba, Holanda con Pocuro, Los Leones con Eliodoro Yáñez, Tobalaba con El Bosque</t>
+          <t>Los Leones con Eliodoro Yáñez</t>
         </is>
       </c>
       <c r="S38" t="inlineStr"/>
+      <c r="T38" t="inlineStr">
+        <is>
+          <t>Destruida</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -3217,23 +3303,23 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Comisionado/a</t>
+          <t>Staff</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>Sí, voy con todo 🤑</t>
         </is>
       </c>
       <c r="G39" t="inlineStr"/>
       <c r="H39" t="inlineStr">
         <is>
-          <t>Viernes</t>
+          <t>Viernes, Sábado</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>Viernes</t>
+          <t>Viernes, Sábado</t>
         </is>
       </c>
       <c r="J39" t="inlineStr">
@@ -3241,35 +3327,32 @@
           <t>Viernes</t>
         </is>
       </c>
-      <c r="K39" t="inlineStr">
-        <is>
-          <t>Viernes</t>
-        </is>
-      </c>
-      <c r="L39" t="inlineStr">
-        <is>
-          <t>Viernes</t>
-        </is>
-      </c>
-      <c r="M39" t="inlineStr">
-        <is>
-          <t>Viernes</t>
-        </is>
-      </c>
+      <c r="K39" t="inlineStr"/>
+      <c r="L39" t="inlineStr"/>
+      <c r="M39" t="inlineStr"/>
       <c r="N39" t="inlineStr"/>
       <c r="O39" t="inlineStr"/>
       <c r="P39" t="inlineStr">
         <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="Q39" t="inlineStr">
+        <is>
           <t>2</t>
         </is>
       </c>
-      <c r="Q39" t="inlineStr"/>
       <c r="R39" t="inlineStr">
         <is>
-          <t>Donde me necesiten</t>
+          <t>Los Leones con Eliodoro Yáñez, Holanda con Pocuro</t>
         </is>
       </c>
       <c r="S39" t="inlineStr"/>
+      <c r="T39" t="inlineStr">
+        <is>
+          <t>Desmejorado</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -3294,47 +3377,72 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Comisionado/a</t>
+          <t>Comisionadx</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>Sí, voy con todo 🤑</t>
         </is>
       </c>
       <c r="G40" t="inlineStr"/>
       <c r="H40" t="inlineStr">
         <is>
-          <t>Sábado</t>
+          <t>Viernes</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>Sábado</t>
+          <t>Viernes, Sábado</t>
         </is>
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>Sábado</t>
-        </is>
-      </c>
-      <c r="K40" t="inlineStr"/>
-      <c r="L40" t="inlineStr"/>
-      <c r="M40" t="inlineStr"/>
-      <c r="N40" t="inlineStr"/>
+          <t>Viernes, Sábado</t>
+        </is>
+      </c>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>Viernes, Sábado</t>
+        </is>
+      </c>
+      <c r="L40" t="inlineStr">
+        <is>
+          <t>Viernes, Sábado</t>
+        </is>
+      </c>
+      <c r="M40" t="inlineStr">
+        <is>
+          <t>Viernes, Sábado</t>
+        </is>
+      </c>
+      <c r="N40" t="inlineStr">
+        <is>
+          <t>Sábado</t>
+        </is>
+      </c>
       <c r="O40" t="inlineStr"/>
-      <c r="P40" t="inlineStr"/>
+      <c r="P40" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="Q40" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>Sin límite</t>
         </is>
       </c>
       <c r="R40" t="inlineStr">
         <is>
-          <t>Tobalaba con El Bosque</t>
+          <t>Donde me necesiten</t>
         </is>
       </c>
       <c r="S40" t="inlineStr"/>
+      <c r="T40" t="inlineStr">
+        <is>
+          <t>Desmejorado</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -3359,47 +3467,60 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Comisionado/a</t>
+          <t>Staff</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="G41" t="inlineStr"/>
-      <c r="H41" t="inlineStr"/>
+          <t>Sí, voy con todo 🤑</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>Sábado</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>Sábado</t>
+        </is>
+      </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>Viernes</t>
+          <t>Sábado</t>
         </is>
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>Viernes</t>
+          <t>Sábado</t>
         </is>
       </c>
       <c r="K41" t="inlineStr">
         <is>
-          <t>Viernes</t>
+          <t>Sábado</t>
         </is>
       </c>
       <c r="L41" t="inlineStr"/>
       <c r="M41" t="inlineStr"/>
       <c r="N41" t="inlineStr"/>
       <c r="O41" t="inlineStr"/>
-      <c r="P41" t="inlineStr">
-        <is>
-          <t>Sin límite</t>
-        </is>
-      </c>
-      <c r="Q41" t="inlineStr"/>
+      <c r="P41" t="inlineStr"/>
+      <c r="Q41" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
       <c r="R41" t="inlineStr">
         <is>
           <t>Donde me necesiten</t>
         </is>
       </c>
       <c r="S41" t="inlineStr"/>
+      <c r="T41" t="inlineStr">
+        <is>
+          <t>Desmejorado</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -3424,12 +3545,12 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Comisionado/a</t>
+          <t>Staff</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>Sí, voy con todo 🤑</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
@@ -3442,26 +3563,10 @@
           <t>Viernes</t>
         </is>
       </c>
-      <c r="I42" t="inlineStr">
-        <is>
-          <t>Viernes</t>
-        </is>
-      </c>
-      <c r="J42" t="inlineStr">
-        <is>
-          <t>Viernes</t>
-        </is>
-      </c>
-      <c r="K42" t="inlineStr">
-        <is>
-          <t>Viernes</t>
-        </is>
-      </c>
-      <c r="L42" t="inlineStr">
-        <is>
-          <t>Viernes</t>
-        </is>
-      </c>
+      <c r="I42" t="inlineStr"/>
+      <c r="J42" t="inlineStr"/>
+      <c r="K42" t="inlineStr"/>
+      <c r="L42" t="inlineStr"/>
       <c r="M42" t="inlineStr"/>
       <c r="N42" t="inlineStr"/>
       <c r="O42" t="inlineStr"/>
@@ -3477,6 +3582,11 @@
         </is>
       </c>
       <c r="S42" t="inlineStr"/>
+      <c r="T42" t="inlineStr">
+        <is>
+          <t>Destruida</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -3501,34 +3611,18 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Familia</t>
+          <t>Comisionadx</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="G43" t="inlineStr">
-        <is>
-          <t>Sábado</t>
-        </is>
-      </c>
-      <c r="H43" t="inlineStr">
-        <is>
-          <t>Sábado</t>
-        </is>
-      </c>
-      <c r="I43" t="inlineStr">
-        <is>
-          <t>Sábado</t>
-        </is>
-      </c>
-      <c r="J43" t="inlineStr">
-        <is>
-          <t>Viernes</t>
-        </is>
-      </c>
+          <t>Sí, voy con todo 🤑</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr"/>
+      <c r="H43" t="inlineStr"/>
+      <c r="I43" t="inlineStr"/>
+      <c r="J43" t="inlineStr"/>
       <c r="K43" t="inlineStr">
         <is>
           <t>Viernes</t>
@@ -3544,24 +3638,33 @@
           <t>Viernes</t>
         </is>
       </c>
-      <c r="N43" t="inlineStr"/>
-      <c r="O43" t="inlineStr"/>
+      <c r="N43" t="inlineStr">
+        <is>
+          <t>Viernes</t>
+        </is>
+      </c>
+      <c r="O43" t="inlineStr">
+        <is>
+          <t>Viernes</t>
+        </is>
+      </c>
       <c r="P43" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="Q43" t="inlineStr">
-        <is>
-          <t>Sin límite</t>
-        </is>
-      </c>
+      <c r="Q43" t="inlineStr"/>
       <c r="R43" t="inlineStr">
         <is>
-          <t>Los Leones con Eliodoro Yáñez</t>
+          <t>Donde me necesiten</t>
         </is>
       </c>
       <c r="S43" t="inlineStr"/>
+      <c r="T43" t="inlineStr">
+        <is>
+          <t>Depauperada</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -3586,67 +3689,60 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Comisionado/a</t>
+          <t>Comisionadx</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="G44" t="inlineStr">
-        <is>
-          <t>Sábado</t>
-        </is>
-      </c>
-      <c r="H44" t="inlineStr">
-        <is>
-          <t>Viernes, Sábado</t>
-        </is>
-      </c>
-      <c r="I44" t="inlineStr">
-        <is>
-          <t>Viernes, Sábado</t>
-        </is>
-      </c>
-      <c r="J44" t="inlineStr">
-        <is>
-          <t>Viernes, Sábado</t>
-        </is>
-      </c>
-      <c r="K44" t="inlineStr">
-        <is>
-          <t>Viernes</t>
-        </is>
-      </c>
+          <t>Sí, voy con todo 🤑</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr"/>
+      <c r="H44" t="inlineStr"/>
+      <c r="I44" t="inlineStr"/>
+      <c r="J44" t="inlineStr"/>
+      <c r="K44" t="inlineStr"/>
       <c r="L44" t="inlineStr">
         <is>
-          <t>Viernes</t>
+          <t>Sábado</t>
         </is>
       </c>
       <c r="M44" t="inlineStr">
         <is>
-          <t>Viernes</t>
-        </is>
-      </c>
-      <c r="N44" t="inlineStr"/>
-      <c r="O44" t="inlineStr"/>
+          <t>Sábado</t>
+        </is>
+      </c>
+      <c r="N44" t="inlineStr">
+        <is>
+          <t>Viernes</t>
+        </is>
+      </c>
+      <c r="O44" t="inlineStr">
+        <is>
+          <t>Viernes</t>
+        </is>
+      </c>
       <c r="P44" t="inlineStr">
         <is>
-          <t>Sin límite</t>
+          <t>3</t>
         </is>
       </c>
       <c r="Q44" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="R44" t="inlineStr">
         <is>
-          <t>Donde me necesiten</t>
+          <t>Francisco Bilbao con Tobalaba, Los Leones con Eliodoro Yáñez, Holanda con Pocuro</t>
         </is>
       </c>
       <c r="S44" t="inlineStr"/>
+      <c r="T44" t="inlineStr">
+        <is>
+          <t>Demacrada</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -3671,59 +3767,52 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Comisionado/a</t>
+          <t>Comisionadx</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="G45" t="inlineStr">
-        <is>
-          <t>Sábado</t>
-        </is>
-      </c>
-      <c r="H45" t="inlineStr">
-        <is>
-          <t>Sábado</t>
-        </is>
-      </c>
+          <t>Sí, voy con todo 🤑</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr"/>
+      <c r="H45" t="inlineStr"/>
       <c r="I45" t="inlineStr">
         <is>
-          <t>Sábado</t>
+          <t>Viernes, Sábado</t>
         </is>
       </c>
       <c r="J45" t="inlineStr">
         <is>
-          <t>Sábado</t>
-        </is>
-      </c>
-      <c r="K45" t="inlineStr">
-        <is>
-          <t>Sábado</t>
-        </is>
-      </c>
-      <c r="L45" t="inlineStr">
-        <is>
-          <t>Sábado</t>
-        </is>
-      </c>
+          <t>Viernes, Sábado</t>
+        </is>
+      </c>
+      <c r="K45" t="inlineStr"/>
+      <c r="L45" t="inlineStr"/>
       <c r="M45" t="inlineStr"/>
       <c r="N45" t="inlineStr"/>
       <c r="O45" t="inlineStr"/>
-      <c r="P45" t="inlineStr"/>
+      <c r="P45" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
       <c r="Q45" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="R45" t="inlineStr">
         <is>
-          <t>Francisco Bilbao con Tobalaba, Holanda con Pocuro, Los Leones con Eliodoro Yáñez</t>
+          <t>Los Leones con Eliodoro Yáñez</t>
         </is>
       </c>
       <c r="S45" t="inlineStr"/>
+      <c r="T45" t="inlineStr">
+        <is>
+          <t>Debilitado</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -3748,43 +3837,52 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Familia</t>
+          <t>Comisionadx</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>Sí, voy con todo 🤑</t>
         </is>
       </c>
       <c r="G46" t="inlineStr"/>
-      <c r="H46" t="inlineStr">
-        <is>
-          <t>Sábado</t>
-        </is>
-      </c>
-      <c r="I46" t="inlineStr">
-        <is>
-          <t>Sábado</t>
-        </is>
-      </c>
+      <c r="H46" t="inlineStr"/>
+      <c r="I46" t="inlineStr"/>
       <c r="J46" t="inlineStr"/>
       <c r="K46" t="inlineStr"/>
       <c r="L46" t="inlineStr"/>
-      <c r="M46" t="inlineStr"/>
-      <c r="N46" t="inlineStr"/>
-      <c r="O46" t="inlineStr"/>
-      <c r="P46" t="inlineStr"/>
-      <c r="Q46" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
+      <c r="M46" t="inlineStr">
+        <is>
+          <t>Viernes</t>
+        </is>
+      </c>
+      <c r="N46" t="inlineStr">
+        <is>
+          <t>Viernes</t>
+        </is>
+      </c>
+      <c r="O46" t="inlineStr">
+        <is>
+          <t>Viernes</t>
+        </is>
+      </c>
+      <c r="P46" t="inlineStr">
+        <is>
+          <t>Sin límite</t>
+        </is>
+      </c>
+      <c r="Q46" t="inlineStr"/>
       <c r="R46" t="inlineStr">
         <is>
-          <t>Donde me necesiten</t>
+          <t>Francisco Bilbao con Tobalaba, Tobalaba con El Bosque</t>
         </is>
       </c>
       <c r="S46" t="inlineStr"/>
+      <c r="T46" t="inlineStr">
+        <is>
+          <t>Demacrada</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -3809,16 +3907,24 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Staff</t>
+          <t>Jefx de comisión</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="G47" t="inlineStr"/>
-      <c r="H47" t="inlineStr"/>
+          <t>Sí, voy con todo 🤑</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>Sábado</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>Sábado</t>
+        </is>
+      </c>
       <c r="I47" t="inlineStr">
         <is>
           <t>Sábado</t>
@@ -3826,50 +3932,31 @@
       </c>
       <c r="J47" t="inlineStr">
         <is>
-          <t>Viernes, Sábado</t>
-        </is>
-      </c>
-      <c r="K47" t="inlineStr">
-        <is>
-          <t>Viernes, Sábado</t>
-        </is>
-      </c>
-      <c r="L47" t="inlineStr">
-        <is>
-          <t>Viernes, Sábado</t>
-        </is>
-      </c>
-      <c r="M47" t="inlineStr">
-        <is>
-          <t>Viernes, Sábado</t>
-        </is>
-      </c>
-      <c r="N47" t="inlineStr">
-        <is>
-          <t>Viernes</t>
-        </is>
-      </c>
-      <c r="O47" t="inlineStr">
-        <is>
-          <t>Viernes</t>
-        </is>
-      </c>
-      <c r="P47" t="inlineStr">
+          <t>Sábado</t>
+        </is>
+      </c>
+      <c r="K47" t="inlineStr"/>
+      <c r="L47" t="inlineStr"/>
+      <c r="M47" t="inlineStr"/>
+      <c r="N47" t="inlineStr"/>
+      <c r="O47" t="inlineStr"/>
+      <c r="P47" t="inlineStr"/>
+      <c r="Q47" t="inlineStr">
         <is>
           <t>Sin límite</t>
         </is>
       </c>
-      <c r="Q47" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
       <c r="R47" t="inlineStr">
         <is>
           <t>Donde me necesiten</t>
         </is>
       </c>
       <c r="S47" t="inlineStr"/>
+      <c r="T47" t="inlineStr">
+        <is>
+          <t>Desmedrado</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -3894,27 +3981,68 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Comisionado/a</t>
+          <t>Staff</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí, voy con todo 🤑</t>
         </is>
       </c>
       <c r="G48" t="inlineStr"/>
-      <c r="H48" t="inlineStr"/>
-      <c r="I48" t="inlineStr"/>
-      <c r="J48" t="inlineStr"/>
-      <c r="K48" t="inlineStr"/>
-      <c r="L48" t="inlineStr"/>
-      <c r="M48" t="inlineStr"/>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>Sábado</t>
+        </is>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>Sábado</t>
+        </is>
+      </c>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>Sábado</t>
+        </is>
+      </c>
+      <c r="K48" t="inlineStr">
+        <is>
+          <t>Viernes, Sábado</t>
+        </is>
+      </c>
+      <c r="L48" t="inlineStr">
+        <is>
+          <t>Viernes</t>
+        </is>
+      </c>
+      <c r="M48" t="inlineStr">
+        <is>
+          <t>Viernes</t>
+        </is>
+      </c>
       <c r="N48" t="inlineStr"/>
       <c r="O48" t="inlineStr"/>
-      <c r="P48" t="inlineStr"/>
-      <c r="Q48" t="inlineStr"/>
-      <c r="R48" t="inlineStr"/>
+      <c r="P48" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="Q48" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="R48" t="inlineStr">
+        <is>
+          <t>Francisco Bilbao con Tobalaba, Los Leones con Eliodoro Yáñez, Holanda con Pocuro</t>
+        </is>
+      </c>
       <c r="S48" t="inlineStr"/>
+      <c r="T48" t="inlineStr">
+        <is>
+          <t>Destruida</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -3939,63 +4067,32 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Familia</t>
+          <t>Comisionadx</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No, odio a financiamiento 😔</t>
         </is>
       </c>
       <c r="G49" t="inlineStr"/>
-      <c r="H49" t="inlineStr">
-        <is>
-          <t>Viernes, Sábado</t>
-        </is>
-      </c>
-      <c r="I49" t="inlineStr">
-        <is>
-          <t>Viernes, Sábado</t>
-        </is>
-      </c>
-      <c r="J49" t="inlineStr">
-        <is>
-          <t>Viernes, Sábado</t>
-        </is>
-      </c>
-      <c r="K49" t="inlineStr">
-        <is>
-          <t>Viernes</t>
-        </is>
-      </c>
-      <c r="L49" t="inlineStr">
-        <is>
-          <t>Viernes</t>
-        </is>
-      </c>
-      <c r="M49" t="inlineStr">
-        <is>
-          <t>Viernes</t>
-        </is>
-      </c>
+      <c r="H49" t="inlineStr"/>
+      <c r="I49" t="inlineStr"/>
+      <c r="J49" t="inlineStr"/>
+      <c r="K49" t="inlineStr"/>
+      <c r="L49" t="inlineStr"/>
+      <c r="M49" t="inlineStr"/>
       <c r="N49" t="inlineStr"/>
       <c r="O49" t="inlineStr"/>
-      <c r="P49" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="Q49" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="R49" t="inlineStr">
-        <is>
-          <t>Holanda con Pocuro</t>
-        </is>
-      </c>
+      <c r="P49" t="inlineStr"/>
+      <c r="Q49" t="inlineStr"/>
+      <c r="R49" t="inlineStr"/>
       <c r="S49" t="inlineStr"/>
+      <c r="T49" t="inlineStr">
+        <is>
+          <t>Depauperada</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -4020,16 +4117,20 @@
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Staff</t>
+          <t>Comisionadx</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>Sí, voy con todo 🤑</t>
         </is>
       </c>
       <c r="G50" t="inlineStr"/>
-      <c r="H50" t="inlineStr"/>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>Viernes</t>
+        </is>
+      </c>
       <c r="I50" t="inlineStr">
         <is>
           <t>Viernes</t>
@@ -4037,42 +4138,55 @@
       </c>
       <c r="J50" t="inlineStr">
         <is>
-          <t>Viernes</t>
+          <t>Viernes, Sábado</t>
         </is>
       </c>
       <c r="K50" t="inlineStr">
         <is>
-          <t>Viernes</t>
+          <t>Sábado</t>
         </is>
       </c>
       <c r="L50" t="inlineStr">
         <is>
-          <t>Viernes</t>
+          <t>Sábado</t>
         </is>
       </c>
       <c r="M50" t="inlineStr">
         <is>
-          <t>Viernes</t>
+          <t>Sábado</t>
         </is>
       </c>
       <c r="N50" t="inlineStr">
         <is>
-          <t>Viernes</t>
-        </is>
-      </c>
-      <c r="O50" t="inlineStr"/>
+          <t>Sábado</t>
+        </is>
+      </c>
+      <c r="O50" t="inlineStr">
+        <is>
+          <t>Sábado</t>
+        </is>
+      </c>
       <c r="P50" t="inlineStr">
         <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="Q50" t="inlineStr"/>
+          <t>Sin límite</t>
+        </is>
+      </c>
+      <c r="Q50" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
       <c r="R50" t="inlineStr">
         <is>
-          <t>Donde me necesiten</t>
+          <t>Tobalaba con El Bosque, Los Leones con Eliodoro Yáñez, Francisco Bilbao con Tobalaba</t>
         </is>
       </c>
       <c r="S50" t="inlineStr"/>
+      <c r="T50" t="inlineStr">
+        <is>
+          <t>Debilitado</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -4097,27 +4211,52 @@
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Comisionado/a</t>
+          <t>Comisionadx</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí, voy con todo 🤑</t>
         </is>
       </c>
       <c r="G51" t="inlineStr"/>
-      <c r="H51" t="inlineStr"/>
-      <c r="I51" t="inlineStr"/>
-      <c r="J51" t="inlineStr"/>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>Viernes</t>
+        </is>
+      </c>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>Viernes</t>
+        </is>
+      </c>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>Viernes</t>
+        </is>
+      </c>
       <c r="K51" t="inlineStr"/>
       <c r="L51" t="inlineStr"/>
       <c r="M51" t="inlineStr"/>
       <c r="N51" t="inlineStr"/>
       <c r="O51" t="inlineStr"/>
-      <c r="P51" t="inlineStr"/>
+      <c r="P51" t="inlineStr">
+        <is>
+          <t>Sin límite</t>
+        </is>
+      </c>
       <c r="Q51" t="inlineStr"/>
-      <c r="R51" t="inlineStr"/>
+      <c r="R51" t="inlineStr">
+        <is>
+          <t>Donde me necesiten</t>
+        </is>
+      </c>
       <c r="S51" t="inlineStr"/>
+      <c r="T51" t="inlineStr">
+        <is>
+          <t>Depauperada</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -4142,25 +4281,37 @@
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Staff</t>
+          <t>Comisionadx</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="G52" t="inlineStr"/>
-      <c r="H52" t="inlineStr"/>
-      <c r="I52" t="inlineStr"/>
+          <t>Sí, voy con todo 🤑</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>Sábado</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>Sábado</t>
+        </is>
+      </c>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>Sábado</t>
+        </is>
+      </c>
       <c r="J52" t="inlineStr">
         <is>
-          <t>Viernes</t>
+          <t>Viernes, Sábado</t>
         </is>
       </c>
       <c r="K52" t="inlineStr">
         <is>
-          <t>Viernes</t>
+          <t>Viernes, Sábado</t>
         </is>
       </c>
       <c r="L52" t="inlineStr">
@@ -4185,16 +4336,25 @@
       </c>
       <c r="P52" t="inlineStr">
         <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="Q52" t="inlineStr">
+        <is>
           <t>3</t>
         </is>
       </c>
-      <c r="Q52" t="inlineStr"/>
       <c r="R52" t="inlineStr">
         <is>
-          <t>Tobalaba con El Bosque, Los Leones con Eliodoro Yáñez, Francisco Bilbao con Tobalaba</t>
+          <t>Donde me necesiten</t>
         </is>
       </c>
       <c r="S52" t="inlineStr"/>
+      <c r="T52" t="inlineStr">
+        <is>
+          <t>Demacrada</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -4219,38 +4379,38 @@
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Comisionado/a</t>
+          <t>Staff</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>Sí, voy con todo 🤑</t>
         </is>
       </c>
       <c r="G53" t="inlineStr"/>
-      <c r="H53" t="inlineStr">
-        <is>
-          <t>Viernes</t>
-        </is>
-      </c>
-      <c r="I53" t="inlineStr">
-        <is>
-          <t>Viernes</t>
-        </is>
-      </c>
+      <c r="H53" t="inlineStr"/>
+      <c r="I53" t="inlineStr"/>
       <c r="J53" t="inlineStr">
         <is>
           <t>Viernes</t>
         </is>
       </c>
-      <c r="K53" t="inlineStr"/>
-      <c r="L53" t="inlineStr"/>
+      <c r="K53" t="inlineStr">
+        <is>
+          <t>Viernes</t>
+        </is>
+      </c>
+      <c r="L53" t="inlineStr">
+        <is>
+          <t>Viernes</t>
+        </is>
+      </c>
       <c r="M53" t="inlineStr"/>
       <c r="N53" t="inlineStr"/>
       <c r="O53" t="inlineStr"/>
       <c r="P53" t="inlineStr">
         <is>
-          <t>Sin límite</t>
+          <t>1</t>
         </is>
       </c>
       <c r="Q53" t="inlineStr"/>
@@ -4260,6 +4420,11 @@
         </is>
       </c>
       <c r="S53" t="inlineStr"/>
+      <c r="T53" t="inlineStr">
+        <is>
+          <t>Debilitado</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -4284,55 +4449,48 @@
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Comisionado/a</t>
+          <t>Comisionadx</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>Sí, voy con todo 🤑</t>
         </is>
       </c>
       <c r="G54" t="inlineStr"/>
       <c r="H54" t="inlineStr"/>
       <c r="I54" t="inlineStr"/>
       <c r="J54" t="inlineStr"/>
-      <c r="K54" t="inlineStr">
-        <is>
-          <t>Viernes</t>
-        </is>
-      </c>
-      <c r="L54" t="inlineStr">
-        <is>
-          <t>Viernes</t>
-        </is>
-      </c>
+      <c r="K54" t="inlineStr"/>
+      <c r="L54" t="inlineStr"/>
       <c r="M54" t="inlineStr">
         <is>
-          <t>Viernes</t>
+          <t>Sábado</t>
         </is>
       </c>
       <c r="N54" t="inlineStr">
         <is>
-          <t>Viernes</t>
-        </is>
-      </c>
-      <c r="O54" t="inlineStr">
-        <is>
-          <t>Viernes</t>
-        </is>
-      </c>
-      <c r="P54" t="inlineStr">
-        <is>
-          <t>Sin límite</t>
-        </is>
-      </c>
-      <c r="Q54" t="inlineStr"/>
+          <t>Sábado</t>
+        </is>
+      </c>
+      <c r="O54" t="inlineStr"/>
+      <c r="P54" t="inlineStr"/>
+      <c r="Q54" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
       <c r="R54" t="inlineStr">
         <is>
-          <t>Donde me necesiten</t>
+          <t>Holanda con Pocuro, Tobalaba con El Bosque, Francisco Bilbao con Tobalaba, Los Leones con Eliodoro Yáñez</t>
         </is>
       </c>
       <c r="S54" t="inlineStr"/>
+      <c r="T54" t="inlineStr">
+        <is>
+          <t>Demacrada</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -4357,47 +4515,48 @@
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Comisionado/a</t>
+          <t>Comisionadx</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>Sí, voy con todo 🤑</t>
         </is>
       </c>
       <c r="G55" t="inlineStr"/>
       <c r="H55" t="inlineStr"/>
       <c r="I55" t="inlineStr"/>
       <c r="J55" t="inlineStr"/>
-      <c r="K55" t="inlineStr">
-        <is>
-          <t>Sábado</t>
-        </is>
-      </c>
-      <c r="L55" t="inlineStr">
-        <is>
-          <t>Sábado</t>
-        </is>
-      </c>
+      <c r="K55" t="inlineStr"/>
+      <c r="L55" t="inlineStr"/>
       <c r="M55" t="inlineStr">
         <is>
-          <t>Sábado</t>
-        </is>
-      </c>
-      <c r="N55" t="inlineStr"/>
+          <t>Viernes</t>
+        </is>
+      </c>
+      <c r="N55" t="inlineStr">
+        <is>
+          <t>Viernes</t>
+        </is>
+      </c>
       <c r="O55" t="inlineStr"/>
-      <c r="P55" t="inlineStr"/>
-      <c r="Q55" t="inlineStr">
-        <is>
-          <t>Sin límite</t>
-        </is>
-      </c>
+      <c r="P55" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="Q55" t="inlineStr"/>
       <c r="R55" t="inlineStr">
         <is>
-          <t>Holanda con Pocuro, Tobalaba con El Bosque</t>
+          <t>Donde me necesiten</t>
         </is>
       </c>
       <c r="S55" t="inlineStr"/>
+      <c r="T55" t="inlineStr">
+        <is>
+          <t>Debilitado</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -4427,7 +4586,7 @@
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No, odio a financiamiento 😔</t>
         </is>
       </c>
       <c r="G56" t="inlineStr"/>
@@ -4435,38 +4594,19 @@
       <c r="I56" t="inlineStr"/>
       <c r="J56" t="inlineStr"/>
       <c r="K56" t="inlineStr"/>
-      <c r="L56" t="inlineStr">
-        <is>
-          <t>Viernes</t>
-        </is>
-      </c>
-      <c r="M56" t="inlineStr">
-        <is>
-          <t>Viernes, Sábado</t>
-        </is>
-      </c>
-      <c r="N56" t="inlineStr">
-        <is>
-          <t>Sábado</t>
-        </is>
-      </c>
+      <c r="L56" t="inlineStr"/>
+      <c r="M56" t="inlineStr"/>
+      <c r="N56" t="inlineStr"/>
       <c r="O56" t="inlineStr"/>
-      <c r="P56" t="inlineStr">
-        <is>
-          <t>Sin límite</t>
-        </is>
-      </c>
-      <c r="Q56" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="R56" t="inlineStr">
-        <is>
-          <t>Holanda con Pocuro, Tobalaba con El Bosque, Francisco Bilbao con Tobalaba, Los Leones con Eliodoro Yáñez</t>
-        </is>
-      </c>
+      <c r="P56" t="inlineStr"/>
+      <c r="Q56" t="inlineStr"/>
+      <c r="R56" t="inlineStr"/>
       <c r="S56" t="inlineStr"/>
+      <c r="T56" t="inlineStr">
+        <is>
+          <t>Destruida</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -4491,19 +4631,15 @@
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>Comisionado/a</t>
+          <t>Staff</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="G57" t="inlineStr">
-        <is>
-          <t>Viernes</t>
-        </is>
-      </c>
+          <t>Sí, voy con todo 🤑</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr"/>
       <c r="H57" t="inlineStr">
         <is>
           <t>Viernes</t>
@@ -4511,43 +4647,56 @@
       </c>
       <c r="I57" t="inlineStr">
         <is>
+          <t>Viernes</t>
+        </is>
+      </c>
+      <c r="J57" t="inlineStr">
+        <is>
+          <t>Viernes</t>
+        </is>
+      </c>
+      <c r="K57" t="inlineStr">
+        <is>
+          <t>Viernes</t>
+        </is>
+      </c>
+      <c r="L57" t="inlineStr">
+        <is>
           <t>Viernes, Sábado</t>
         </is>
       </c>
-      <c r="J57" t="inlineStr">
-        <is>
-          <t>Sábado</t>
-        </is>
-      </c>
-      <c r="K57" t="inlineStr">
-        <is>
-          <t>Sábado</t>
-        </is>
-      </c>
-      <c r="L57" t="inlineStr">
-        <is>
-          <t>Sábado</t>
-        </is>
-      </c>
-      <c r="M57" t="inlineStr"/>
-      <c r="N57" t="inlineStr"/>
+      <c r="M57" t="inlineStr">
+        <is>
+          <t>Viernes, Sábado</t>
+        </is>
+      </c>
+      <c r="N57" t="inlineStr">
+        <is>
+          <t>Sábado</t>
+        </is>
+      </c>
       <c r="O57" t="inlineStr"/>
       <c r="P57" t="inlineStr">
         <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="Q57" t="inlineStr">
+        <is>
           <t>Sin límite</t>
         </is>
       </c>
-      <c r="Q57" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
       <c r="R57" t="inlineStr">
         <is>
-          <t>Holanda con Pocuro</t>
+          <t>Francisco Bilbao con Tobalaba, Tobalaba con El Bosque</t>
         </is>
       </c>
       <c r="S57" t="inlineStr"/>
+      <c r="T57" t="inlineStr">
+        <is>
+          <t>Depauperada</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -4572,12 +4721,12 @@
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>Comisionado/a</t>
+          <t>Comisionadx</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No, odio a financiamiento 😔</t>
         </is>
       </c>
       <c r="G58" t="inlineStr"/>
@@ -4586,33 +4735,18 @@
       <c r="J58" t="inlineStr"/>
       <c r="K58" t="inlineStr"/>
       <c r="L58" t="inlineStr"/>
-      <c r="M58" t="inlineStr">
-        <is>
-          <t>Sábado</t>
-        </is>
-      </c>
-      <c r="N58" t="inlineStr">
-        <is>
-          <t>Sábado</t>
-        </is>
-      </c>
-      <c r="O58" t="inlineStr">
-        <is>
-          <t>Sábado</t>
-        </is>
-      </c>
+      <c r="M58" t="inlineStr"/>
+      <c r="N58" t="inlineStr"/>
+      <c r="O58" t="inlineStr"/>
       <c r="P58" t="inlineStr"/>
-      <c r="Q58" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="R58" t="inlineStr">
-        <is>
-          <t>Donde me necesiten</t>
-        </is>
-      </c>
+      <c r="Q58" t="inlineStr"/>
+      <c r="R58" t="inlineStr"/>
       <c r="S58" t="inlineStr"/>
+      <c r="T58" t="inlineStr">
+        <is>
+          <t>Desmejorado</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -4637,25 +4771,17 @@
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>Familia</t>
+          <t>Comisionadx</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>Sí, voy con todo 🤑</t>
         </is>
       </c>
       <c r="G59" t="inlineStr"/>
-      <c r="H59" t="inlineStr">
-        <is>
-          <t>Viernes</t>
-        </is>
-      </c>
-      <c r="I59" t="inlineStr">
-        <is>
-          <t>Viernes</t>
-        </is>
-      </c>
+      <c r="H59" t="inlineStr"/>
+      <c r="I59" t="inlineStr"/>
       <c r="J59" t="inlineStr">
         <is>
           <t>Viernes, Sábado</t>
@@ -4671,25 +4797,42 @@
           <t>Viernes, Sábado</t>
         </is>
       </c>
-      <c r="M59" t="inlineStr"/>
-      <c r="N59" t="inlineStr"/>
-      <c r="O59" t="inlineStr"/>
+      <c r="M59" t="inlineStr">
+        <is>
+          <t>Sábado</t>
+        </is>
+      </c>
+      <c r="N59" t="inlineStr">
+        <is>
+          <t>Sábado</t>
+        </is>
+      </c>
+      <c r="O59" t="inlineStr">
+        <is>
+          <t>Sábado</t>
+        </is>
+      </c>
       <c r="P59" t="inlineStr">
         <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="Q59" t="inlineStr">
+        <is>
           <t>1</t>
         </is>
       </c>
-      <c r="Q59" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
       <c r="R59" t="inlineStr">
         <is>
-          <t>Holanda con Pocuro, Tobalaba con El Bosque, Los Leones con Eliodoro Yáñez</t>
+          <t>Los Leones con Eliodoro Yáñez, Holanda con Pocuro, Francisco Bilbao con Tobalaba</t>
         </is>
       </c>
       <c r="S59" t="inlineStr"/>
+      <c r="T59" t="inlineStr">
+        <is>
+          <t>Depauperada</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -4714,12 +4857,12 @@
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>Familia</t>
+          <t>Staff</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>Sí, voy con todo 🤑</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
@@ -4734,47 +4877,60 @@
       </c>
       <c r="I60" t="inlineStr">
         <is>
+          <t>Sábado</t>
+        </is>
+      </c>
+      <c r="J60" t="inlineStr">
+        <is>
+          <t>Sábado</t>
+        </is>
+      </c>
+      <c r="K60" t="inlineStr">
+        <is>
           <t>Viernes, Sábado</t>
         </is>
       </c>
-      <c r="J60" t="inlineStr">
+      <c r="L60" t="inlineStr">
         <is>
           <t>Viernes, Sábado</t>
         </is>
       </c>
-      <c r="K60" t="inlineStr">
-        <is>
-          <t>Viernes</t>
-        </is>
-      </c>
-      <c r="L60" t="inlineStr">
-        <is>
-          <t>Viernes</t>
-        </is>
-      </c>
       <c r="M60" t="inlineStr">
         <is>
           <t>Viernes</t>
         </is>
       </c>
-      <c r="N60" t="inlineStr"/>
-      <c r="O60" t="inlineStr"/>
+      <c r="N60" t="inlineStr">
+        <is>
+          <t>Viernes</t>
+        </is>
+      </c>
+      <c r="O60" t="inlineStr">
+        <is>
+          <t>Viernes</t>
+        </is>
+      </c>
       <c r="P60" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="Q60" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>Sin límite</t>
         </is>
       </c>
       <c r="R60" t="inlineStr">
         <is>
-          <t>Los Leones con Eliodoro Yáñez, Tobalaba con El Bosque, Holanda con Pocuro</t>
+          <t>Los Leones con Eliodoro Yáñez, Holanda con Pocuro</t>
         </is>
       </c>
       <c r="S60" t="inlineStr"/>
+      <c r="T60" t="inlineStr">
+        <is>
+          <t>Destruida</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -4799,59 +4955,60 @@
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>Staff</t>
+          <t>Comisionadx</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="G61" t="inlineStr">
-        <is>
-          <t>Sábado</t>
-        </is>
-      </c>
-      <c r="H61" t="inlineStr">
-        <is>
-          <t>Sábado</t>
-        </is>
-      </c>
-      <c r="I61" t="inlineStr">
-        <is>
-          <t>Sábado</t>
-        </is>
-      </c>
-      <c r="J61" t="inlineStr">
-        <is>
-          <t>Sábado</t>
-        </is>
-      </c>
+          <t>Sí, voy con todo 🤑</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr"/>
+      <c r="H61" t="inlineStr"/>
+      <c r="I61" t="inlineStr"/>
+      <c r="J61" t="inlineStr"/>
       <c r="K61" t="inlineStr">
         <is>
-          <t>Sábado</t>
+          <t>Viernes</t>
         </is>
       </c>
       <c r="L61" t="inlineStr">
         <is>
-          <t>Sábado</t>
-        </is>
-      </c>
-      <c r="M61" t="inlineStr"/>
-      <c r="N61" t="inlineStr"/>
+          <t>Viernes</t>
+        </is>
+      </c>
+      <c r="M61" t="inlineStr">
+        <is>
+          <t>Viernes, Sábado</t>
+        </is>
+      </c>
+      <c r="N61" t="inlineStr">
+        <is>
+          <t>Sábado</t>
+        </is>
+      </c>
       <c r="O61" t="inlineStr"/>
-      <c r="P61" t="inlineStr"/>
+      <c r="P61" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
       <c r="Q61" t="inlineStr">
         <is>
-          <t>Sin límite</t>
+          <t>2</t>
         </is>
       </c>
       <c r="R61" t="inlineStr">
         <is>
-          <t>Los Leones con Eliodoro Yáñez, Holanda con Pocuro</t>
+          <t>Tobalaba con El Bosque, Francisco Bilbao con Tobalaba</t>
         </is>
       </c>
       <c r="S61" t="inlineStr"/>
+      <c r="T61" t="inlineStr">
+        <is>
+          <t>Desmejorado</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>